<commit_message>
Remove review_reason column from .review files
</commit_message>
<xml_diff>
--- a/output/campaign_Otros_proyectos.review.xlsx
+++ b/output/campaign_Otros_proyectos.review.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G187"/>
+  <dimension ref="A1:F187"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,11 +447,6 @@
           <t>Negocio ID</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>review_reason</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -480,11 +475,6 @@
       <c r="F2" t="n">
         <v>57308478045</v>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>duplicate</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -513,11 +503,6 @@
       <c r="F3" t="n">
         <v>13528427428</v>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>duplicate</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -546,11 +531,6 @@
       <c r="F4" t="n">
         <v>3270775068</v>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>duplicate</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -571,11 +551,6 @@
       <c r="F5" t="n">
         <v/>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -596,11 +571,6 @@
       <c r="F6" t="n">
         <v/>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -621,11 +591,6 @@
       <c r="F7" t="n">
         <v/>
       </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -646,11 +611,6 @@
       <c r="F8" t="n">
         <v/>
       </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -671,11 +631,6 @@
       <c r="F9" t="n">
         <v/>
       </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -696,11 +651,6 @@
       <c r="F10" t="n">
         <v/>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -721,11 +671,6 @@
       <c r="F11" t="n">
         <v/>
       </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -746,11 +691,6 @@
       <c r="F12" t="n">
         <v/>
       </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -771,11 +711,6 @@
       <c r="F13" t="n">
         <v/>
       </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -796,11 +731,6 @@
       <c r="F14" t="n">
         <v/>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -821,11 +751,6 @@
       <c r="F15" t="n">
         <v/>
       </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -846,11 +771,6 @@
       <c r="F16" t="n">
         <v/>
       </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -871,11 +791,6 @@
       <c r="F17" t="n">
         <v/>
       </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -896,11 +811,6 @@
       <c r="F18" t="n">
         <v/>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -921,11 +831,6 @@
       <c r="F19" t="n">
         <v/>
       </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -946,11 +851,6 @@
       <c r="F20" t="n">
         <v/>
       </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -971,11 +871,6 @@
       <c r="F21" t="n">
         <v/>
       </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -996,11 +891,6 @@
       <c r="F22" t="n">
         <v/>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1021,11 +911,6 @@
       <c r="F23" t="n">
         <v/>
       </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1046,11 +931,6 @@
       <c r="F24" t="n">
         <v/>
       </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1071,11 +951,6 @@
       <c r="F25" t="n">
         <v/>
       </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1096,11 +971,6 @@
       <c r="F26" t="n">
         <v/>
       </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1121,11 +991,6 @@
       <c r="F27" t="n">
         <v/>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1146,11 +1011,6 @@
       <c r="F28" t="n">
         <v/>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1171,11 +1031,6 @@
       <c r="F29" t="n">
         <v/>
       </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1196,11 +1051,6 @@
       <c r="F30" t="n">
         <v/>
       </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1221,11 +1071,6 @@
       <c r="F31" t="n">
         <v/>
       </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1246,11 +1091,6 @@
       <c r="F32" t="n">
         <v/>
       </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1271,11 +1111,6 @@
       <c r="F33" t="n">
         <v/>
       </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1296,11 +1131,6 @@
       <c r="F34" t="n">
         <v/>
       </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1321,11 +1151,6 @@
       <c r="F35" t="n">
         <v/>
       </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1346,11 +1171,6 @@
       <c r="F36" t="n">
         <v/>
       </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1371,11 +1191,6 @@
       <c r="F37" t="n">
         <v/>
       </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1396,11 +1211,6 @@
       <c r="F38" t="n">
         <v/>
       </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1421,11 +1231,6 @@
       <c r="F39" t="n">
         <v/>
       </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1446,11 +1251,6 @@
       <c r="F40" t="n">
         <v/>
       </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1471,11 +1271,6 @@
       <c r="F41" t="n">
         <v/>
       </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1496,11 +1291,6 @@
       <c r="F42" t="n">
         <v/>
       </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1521,11 +1311,6 @@
       <c r="F43" t="n">
         <v/>
       </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1546,11 +1331,6 @@
       <c r="F44" t="n">
         <v/>
       </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1571,11 +1351,6 @@
       <c r="F45" t="n">
         <v/>
       </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1596,11 +1371,6 @@
       <c r="F46" t="n">
         <v/>
       </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1621,11 +1391,6 @@
       <c r="F47" t="n">
         <v/>
       </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1646,11 +1411,6 @@
       <c r="F48" t="n">
         <v/>
       </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1671,11 +1431,6 @@
       <c r="F49" t="n">
         <v/>
       </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1696,11 +1451,6 @@
       <c r="F50" t="n">
         <v/>
       </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1721,11 +1471,6 @@
       <c r="F51" t="n">
         <v/>
       </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1746,11 +1491,6 @@
       <c r="F52" t="n">
         <v/>
       </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -1771,11 +1511,6 @@
       <c r="F53" t="n">
         <v/>
       </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -1796,11 +1531,6 @@
       <c r="F54" t="n">
         <v/>
       </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -1821,11 +1551,6 @@
       <c r="F55" t="n">
         <v/>
       </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -1846,11 +1571,6 @@
       <c r="F56" t="n">
         <v/>
       </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -1871,11 +1591,6 @@
       <c r="F57" t="n">
         <v/>
       </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -1896,11 +1611,6 @@
       <c r="F58" t="n">
         <v/>
       </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -1921,11 +1631,6 @@
       <c r="F59" t="n">
         <v/>
       </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -1946,11 +1651,6 @@
       <c r="F60" t="n">
         <v/>
       </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -1971,11 +1671,6 @@
       <c r="F61" t="n">
         <v/>
       </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -1996,11 +1691,6 @@
       <c r="F62" t="n">
         <v/>
       </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -2021,11 +1711,6 @@
       <c r="F63" t="n">
         <v/>
       </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -2046,11 +1731,6 @@
       <c r="F64" t="n">
         <v/>
       </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -2071,11 +1751,6 @@
       <c r="F65" t="n">
         <v/>
       </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -2096,11 +1771,6 @@
       <c r="F66" t="n">
         <v/>
       </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -2121,11 +1791,6 @@
       <c r="F67" t="n">
         <v/>
       </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -2146,11 +1811,6 @@
       <c r="F68" t="n">
         <v/>
       </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -2171,11 +1831,6 @@
       <c r="F69" t="n">
         <v/>
       </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -2196,11 +1851,6 @@
       <c r="F70" t="n">
         <v/>
       </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -2221,11 +1871,6 @@
       <c r="F71" t="n">
         <v/>
       </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -2246,11 +1891,6 @@
       <c r="F72" t="n">
         <v/>
       </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -2271,11 +1911,6 @@
       <c r="F73" t="n">
         <v/>
       </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -2296,11 +1931,6 @@
       <c r="F74" t="n">
         <v/>
       </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -2321,11 +1951,6 @@
       <c r="F75" t="n">
         <v/>
       </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -2346,11 +1971,6 @@
       <c r="F76" t="n">
         <v/>
       </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -2371,11 +1991,6 @@
       <c r="F77" t="n">
         <v/>
       </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -2396,11 +2011,6 @@
       <c r="F78" t="n">
         <v/>
       </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -2421,11 +2031,6 @@
       <c r="F79" t="n">
         <v/>
       </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -2446,11 +2051,6 @@
       <c r="F80" t="n">
         <v/>
       </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -2471,11 +2071,6 @@
       <c r="F81" t="n">
         <v/>
       </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -2496,11 +2091,6 @@
       <c r="F82" t="n">
         <v/>
       </c>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -2521,11 +2111,6 @@
       <c r="F83" t="n">
         <v/>
       </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -2546,11 +2131,6 @@
       <c r="F84" t="n">
         <v/>
       </c>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -2571,11 +2151,6 @@
       <c r="F85" t="n">
         <v/>
       </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -2596,11 +2171,6 @@
       <c r="F86" t="n">
         <v/>
       </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -2621,11 +2191,6 @@
       <c r="F87" t="n">
         <v/>
       </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -2646,11 +2211,6 @@
       <c r="F88" t="n">
         <v/>
       </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -2671,11 +2231,6 @@
       <c r="F89" t="n">
         <v/>
       </c>
-      <c r="G89" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -2696,11 +2251,6 @@
       <c r="F90" t="n">
         <v/>
       </c>
-      <c r="G90" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -2721,11 +2271,6 @@
       <c r="F91" t="n">
         <v/>
       </c>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -2746,11 +2291,6 @@
       <c r="F92" t="n">
         <v/>
       </c>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -2771,11 +2311,6 @@
       <c r="F93" t="n">
         <v/>
       </c>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -2796,11 +2331,6 @@
       <c r="F94" t="n">
         <v/>
       </c>
-      <c r="G94" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -2821,11 +2351,6 @@
       <c r="F95" t="n">
         <v/>
       </c>
-      <c r="G95" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -2846,11 +2371,6 @@
       <c r="F96" t="n">
         <v/>
       </c>
-      <c r="G96" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -2871,11 +2391,6 @@
       <c r="F97" t="n">
         <v/>
       </c>
-      <c r="G97" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -2896,11 +2411,6 @@
       <c r="F98" t="n">
         <v/>
       </c>
-      <c r="G98" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -2921,11 +2431,6 @@
       <c r="F99" t="n">
         <v/>
       </c>
-      <c r="G99" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -2946,11 +2451,6 @@
       <c r="F100" t="n">
         <v/>
       </c>
-      <c r="G100" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -2971,11 +2471,6 @@
       <c r="F101" t="n">
         <v/>
       </c>
-      <c r="G101" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -2996,11 +2491,6 @@
       <c r="F102" t="n">
         <v/>
       </c>
-      <c r="G102" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -3021,11 +2511,6 @@
       <c r="F103" t="n">
         <v/>
       </c>
-      <c r="G103" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -3046,11 +2531,6 @@
       <c r="F104" t="n">
         <v/>
       </c>
-      <c r="G104" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -3071,11 +2551,6 @@
       <c r="F105" t="n">
         <v/>
       </c>
-      <c r="G105" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -3096,11 +2571,6 @@
       <c r="F106" t="n">
         <v/>
       </c>
-      <c r="G106" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -3121,11 +2591,6 @@
       <c r="F107" t="n">
         <v/>
       </c>
-      <c r="G107" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -3146,11 +2611,6 @@
       <c r="F108" t="n">
         <v/>
       </c>
-      <c r="G108" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -3171,11 +2631,6 @@
       <c r="F109" t="n">
         <v/>
       </c>
-      <c r="G109" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -3196,11 +2651,6 @@
       <c r="F110" t="n">
         <v/>
       </c>
-      <c r="G110" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -3221,11 +2671,6 @@
       <c r="F111" t="n">
         <v/>
       </c>
-      <c r="G111" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -3246,11 +2691,6 @@
       <c r="F112" t="n">
         <v/>
       </c>
-      <c r="G112" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -3271,11 +2711,6 @@
       <c r="F113" t="n">
         <v/>
       </c>
-      <c r="G113" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -3296,11 +2731,6 @@
       <c r="F114" t="n">
         <v/>
       </c>
-      <c r="G114" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -3321,11 +2751,6 @@
       <c r="F115" t="n">
         <v/>
       </c>
-      <c r="G115" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -3346,11 +2771,6 @@
       <c r="F116" t="n">
         <v/>
       </c>
-      <c r="G116" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -3371,11 +2791,6 @@
       <c r="F117" t="n">
         <v/>
       </c>
-      <c r="G117" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -3396,11 +2811,6 @@
       <c r="F118" t="n">
         <v/>
       </c>
-      <c r="G118" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -3421,11 +2831,6 @@
       <c r="F119" t="n">
         <v/>
       </c>
-      <c r="G119" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -3446,11 +2851,6 @@
       <c r="F120" t="n">
         <v/>
       </c>
-      <c r="G120" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -3471,11 +2871,6 @@
       <c r="F121" t="n">
         <v/>
       </c>
-      <c r="G121" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -3496,11 +2891,6 @@
       <c r="F122" t="n">
         <v/>
       </c>
-      <c r="G122" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -3521,11 +2911,6 @@
       <c r="F123" t="n">
         <v/>
       </c>
-      <c r="G123" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -3546,11 +2931,6 @@
       <c r="F124" t="n">
         <v/>
       </c>
-      <c r="G124" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -3571,11 +2951,6 @@
       <c r="F125" t="n">
         <v/>
       </c>
-      <c r="G125" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -3596,11 +2971,6 @@
       <c r="F126" t="n">
         <v/>
       </c>
-      <c r="G126" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -3621,11 +2991,6 @@
       <c r="F127" t="n">
         <v/>
       </c>
-      <c r="G127" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -3646,11 +3011,6 @@
       <c r="F128" t="n">
         <v/>
       </c>
-      <c r="G128" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -3671,11 +3031,6 @@
       <c r="F129" t="n">
         <v/>
       </c>
-      <c r="G129" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -3696,11 +3051,6 @@
       <c r="F130" t="n">
         <v/>
       </c>
-      <c r="G130" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -3721,11 +3071,6 @@
       <c r="F131" t="n">
         <v/>
       </c>
-      <c r="G131" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -3746,11 +3091,6 @@
       <c r="F132" t="n">
         <v/>
       </c>
-      <c r="G132" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -3771,11 +3111,6 @@
       <c r="F133" t="n">
         <v/>
       </c>
-      <c r="G133" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -3796,11 +3131,6 @@
       <c r="F134" t="n">
         <v/>
       </c>
-      <c r="G134" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -3821,11 +3151,6 @@
       <c r="F135" t="n">
         <v/>
       </c>
-      <c r="G135" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -3846,11 +3171,6 @@
       <c r="F136" t="n">
         <v/>
       </c>
-      <c r="G136" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -3871,11 +3191,6 @@
       <c r="F137" t="n">
         <v/>
       </c>
-      <c r="G137" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -3896,11 +3211,6 @@
       <c r="F138" t="n">
         <v/>
       </c>
-      <c r="G138" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -3921,11 +3231,6 @@
       <c r="F139" t="n">
         <v/>
       </c>
-      <c r="G139" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -3946,11 +3251,6 @@
       <c r="F140" t="n">
         <v/>
       </c>
-      <c r="G140" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -3971,11 +3271,6 @@
       <c r="F141" t="n">
         <v/>
       </c>
-      <c r="G141" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -3996,11 +3291,6 @@
       <c r="F142" t="n">
         <v/>
       </c>
-      <c r="G142" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -4021,11 +3311,6 @@
       <c r="F143" t="n">
         <v/>
       </c>
-      <c r="G143" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -4046,11 +3331,6 @@
       <c r="F144" t="n">
         <v/>
       </c>
-      <c r="G144" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -4071,11 +3351,6 @@
       <c r="F145" t="n">
         <v/>
       </c>
-      <c r="G145" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -4096,11 +3371,6 @@
       <c r="F146" t="n">
         <v/>
       </c>
-      <c r="G146" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -4121,11 +3391,6 @@
       <c r="F147" t="n">
         <v/>
       </c>
-      <c r="G147" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -4146,11 +3411,6 @@
       <c r="F148" t="n">
         <v/>
       </c>
-      <c r="G148" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -4171,11 +3431,6 @@
       <c r="F149" t="n">
         <v/>
       </c>
-      <c r="G149" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -4196,11 +3451,6 @@
       <c r="F150" t="n">
         <v/>
       </c>
-      <c r="G150" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -4221,11 +3471,6 @@
       <c r="F151" t="n">
         <v/>
       </c>
-      <c r="G151" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -4246,11 +3491,6 @@
       <c r="F152" t="n">
         <v/>
       </c>
-      <c r="G152" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -4271,11 +3511,6 @@
       <c r="F153" t="n">
         <v/>
       </c>
-      <c r="G153" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -4296,11 +3531,6 @@
       <c r="F154" t="n">
         <v/>
       </c>
-      <c r="G154" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -4321,11 +3551,6 @@
       <c r="F155" t="n">
         <v/>
       </c>
-      <c r="G155" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -4346,11 +3571,6 @@
       <c r="F156" t="n">
         <v/>
       </c>
-      <c r="G156" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -4371,11 +3591,6 @@
       <c r="F157" t="n">
         <v/>
       </c>
-      <c r="G157" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -4396,11 +3611,6 @@
       <c r="F158" t="n">
         <v/>
       </c>
-      <c r="G158" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -4421,11 +3631,6 @@
       <c r="F159" t="n">
         <v/>
       </c>
-      <c r="G159" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -4446,11 +3651,6 @@
       <c r="F160" t="n">
         <v/>
       </c>
-      <c r="G160" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -4471,11 +3671,6 @@
       <c r="F161" t="n">
         <v/>
       </c>
-      <c r="G161" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="162">
       <c r="A162" t="n">
@@ -4496,11 +3691,6 @@
       <c r="F162" t="n">
         <v/>
       </c>
-      <c r="G162" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="163">
       <c r="A163" t="n">
@@ -4521,11 +3711,6 @@
       <c r="F163" t="n">
         <v/>
       </c>
-      <c r="G163" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="164">
       <c r="A164" t="n">
@@ -4546,11 +3731,6 @@
       <c r="F164" t="n">
         <v/>
       </c>
-      <c r="G164" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="165">
       <c r="A165" t="n">
@@ -4571,11 +3751,6 @@
       <c r="F165" t="n">
         <v/>
       </c>
-      <c r="G165" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="166">
       <c r="A166" t="n">
@@ -4596,11 +3771,6 @@
       <c r="F166" t="n">
         <v/>
       </c>
-      <c r="G166" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="167">
       <c r="A167" t="n">
@@ -4621,11 +3791,6 @@
       <c r="F167" t="n">
         <v/>
       </c>
-      <c r="G167" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="168">
       <c r="A168" t="n">
@@ -4646,11 +3811,6 @@
       <c r="F168" t="n">
         <v/>
       </c>
-      <c r="G168" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="169">
       <c r="A169" t="n">
@@ -4671,11 +3831,6 @@
       <c r="F169" t="n">
         <v/>
       </c>
-      <c r="G169" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="170">
       <c r="A170" t="n">
@@ -4696,11 +3851,6 @@
       <c r="F170" t="n">
         <v/>
       </c>
-      <c r="G170" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="171">
       <c r="A171" t="n">
@@ -4721,11 +3871,6 @@
       <c r="F171" t="n">
         <v/>
       </c>
-      <c r="G171" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="172">
       <c r="A172" t="n">
@@ -4746,11 +3891,6 @@
       <c r="F172" t="n">
         <v/>
       </c>
-      <c r="G172" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="173">
       <c r="A173" t="n">
@@ -4771,11 +3911,6 @@
       <c r="F173" t="n">
         <v/>
       </c>
-      <c r="G173" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="174">
       <c r="A174" t="n">
@@ -4796,11 +3931,6 @@
       <c r="F174" t="n">
         <v/>
       </c>
-      <c r="G174" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="175">
       <c r="A175" t="n">
@@ -4821,11 +3951,6 @@
       <c r="F175" t="n">
         <v/>
       </c>
-      <c r="G175" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="176">
       <c r="A176" t="n">
@@ -4846,11 +3971,6 @@
       <c r="F176" t="n">
         <v/>
       </c>
-      <c r="G176" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="177">
       <c r="A177" t="n">
@@ -4871,11 +3991,6 @@
       <c r="F177" t="n">
         <v/>
       </c>
-      <c r="G177" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="178">
       <c r="A178" t="n">
@@ -4896,11 +4011,6 @@
       <c r="F178" t="n">
         <v/>
       </c>
-      <c r="G178" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="179">
       <c r="A179" t="n">
@@ -4921,11 +4031,6 @@
       <c r="F179" t="n">
         <v/>
       </c>
-      <c r="G179" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -4946,11 +4051,6 @@
       <c r="F180" t="n">
         <v/>
       </c>
-      <c r="G180" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="181">
       <c r="A181" t="n">
@@ -4971,11 +4071,6 @@
       <c r="F181" t="n">
         <v/>
       </c>
-      <c r="G181" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -4996,11 +4091,6 @@
       <c r="F182" t="n">
         <v/>
       </c>
-      <c r="G182" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="183">
       <c r="A183" t="n">
@@ -5021,11 +4111,6 @@
       <c r="F183" t="n">
         <v/>
       </c>
-      <c r="G183" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="184">
       <c r="A184" t="n">
@@ -5046,11 +4131,6 @@
       <c r="F184" t="n">
         <v/>
       </c>
-      <c r="G184" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="185">
       <c r="A185" t="n">
@@ -5071,11 +4151,6 @@
       <c r="F185" t="n">
         <v/>
       </c>
-      <c r="G185" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="186">
       <c r="A186" t="n">
@@ -5096,11 +4171,6 @@
       <c r="F186" t="n">
         <v/>
       </c>
-      <c r="G186" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
-      </c>
     </row>
     <row r="187">
       <c r="A187" t="n">
@@ -5120,11 +4190,6 @@
       </c>
       <c r="F187" t="n">
         <v/>
-      </c>
-      <c r="G187" t="inlineStr">
-        <is>
-          <t>empty</t>
-        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Clean rewrite: fix nombre_cliente, hubspot_deal_id, phone normalization
- nombre_cliente: concatenates Nombre + Apellidos with one space
- hubspot_deal_id: full integer string, no scientific notation
- Phone normalization: valid digits only in output; invalid/ambiguous
  phones quarantined to .review files as the word 'review'
- Duplicates dropped silently
</commit_message>
<xml_diff>
--- a/output/campaign_Otros_proyectos.review.xlsx
+++ b/output/campaign_Otros_proyectos.review.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A187"/>
+  <dimension ref="A1:A184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1704,27 +1704,6 @@
         </is>
       </c>
     </row>
-    <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t>review</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>